<commit_message>
docs: demonstrate deterministic numeric writing
</commit_message>
<xml_diff>
--- a/samples/polars_dataframe_output.xlsx
+++ b/samples/polars_dataframe_output.xlsx
@@ -526,13 +526,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -543,17 +544,19 @@
       </c>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
-      <c r="D1" s="3" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="3" t="n"/>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>The adapter preserves row order and column names; template syntax remains library-neutral.</t>
+          <t>Polars computes the Decimal result column before the adapter renders numeric cells.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
-      <c r="D2" s="3" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -576,6 +579,11 @@
           <t>Optional</t>
         </is>
       </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Computed amount</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -584,13 +592,16 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>1250</v>
+        <v>1250.0</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>46253</v>
+        <v>46253.0</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>1</v>
+        <v>1.0</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>1312.5</v>
       </c>
     </row>
     <row r="6">
@@ -600,12 +611,15 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>350</v>
+        <v>350.0</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>46254</v>
+        <v>46254.0</v>
       </c>
       <c r="D6" s="5" t="n"/>
+      <c r="E6" s="6" t="n">
+        <v>367.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -614,12 +628,15 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>875</v>
+        <v>875.0</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>46255</v>
+        <v>46255.0</v>
       </c>
       <c r="D7" s="5" t="n"/>
+      <c r="E7" s="6" t="n">
+        <v>918.75</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -629,13 +646,14 @@
       </c>
       <c r="B8" s="2" t="n"/>
       <c r="C8" s="2" t="n"/>
-      <c r="D8" s="3" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A8:E8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>